<commit_message>
Write Remark as bullet points instead of one run-on paragraph
Each flag (merged mode, cause/mode mismatch, ambiguity, plant-vs-AI
disagreement, duplicate cause) now gets its own bullet line so nothing
gets lost reading a multi-flag row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions_gpt4omini.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions_gpt4omini.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -2605,7 +2605,11 @@
       </c>
       <c r="AW18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage; it aligns with a wrong-variant selection/installation failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>- Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet.
+- Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage; it aligns with a wrong-variant selection/installation failure mode instead.
+- Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing.
+- AI severity (8) differs from plant-recorded (5) - review recommended.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2754,7 +2758,10 @@
       </c>
       <c r="AW20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>- Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet.
+- Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing.
+- AI severity (8) differs from plant-recorded (5) - review recommended.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2909,7 @@
       <c r="AV22" s="223" t="inlineStr"/>
       <c r="AW22" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3066,7 @@
       <c r="AV24" s="223" t="inlineStr"/>
       <c r="AW24" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3235,7 @@
       </c>
       <c r="AW26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet.</t>
+          <t>- Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet.</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3395,7 @@
       <c r="AV28" s="223" t="inlineStr"/>
       <c r="AW28" s="223" t="inlineStr">
         <is>
-          <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3485,8 @@
       </c>
       <c r="AW29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>- Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>

</xml_diff>